<commit_message>
Regenerate employee upload templates from the 1.0.9 desktop build.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/resources/templates/employee_salary_upload_template.xlsx
+++ b/resources/templates/employee_salary_upload_template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="41">
   <si>
     <t>employee_number</t>
   </si>
@@ -53,6 +53,9 @@
     <t>is_above_minimum_wage_earner</t>
   </si>
   <si>
+    <t>is_fixed_rate</t>
+  </si>
+  <si>
     <t>basic_taxable</t>
   </si>
   <si>
@@ -99,6 +102,9 @@
   </si>
   <si>
     <t>Is Above Minimum Wage Earner (yes/no)</t>
+  </si>
+  <si>
+    <t>Is Fixed Rate (yes/no)</t>
   </si>
   <si>
     <t>Basic Income Taxable</t>
@@ -472,10 +478,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:P154"/>
+  <dimension ref="A1:Q154"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:17">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -524,84 +530,90 @@
       <c r="P1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:16">
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="M2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="O2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16">
+        <v>32</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G3" t="s">
         <v>35</v>
       </c>
-      <c r="F3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G3" t="s">
-        <v>33</v>
-      </c>
       <c r="J3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16">
+        <v>39</v>
+      </c>
+      <c r="N3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -618,8 +630,9 @@
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
       <c r="P4" s="1"/>
-    </row>
-    <row r="5" spans="1:16">
+      <c r="Q4" s="1"/>
+    </row>
+    <row r="5" spans="1:17">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -636,8 +649,9 @@
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
-    </row>
-    <row r="6" spans="1:16">
+      <c r="Q5" s="1"/>
+    </row>
+    <row r="6" spans="1:17">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -654,8 +668,9 @@
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
-    </row>
-    <row r="7" spans="1:16">
+      <c r="Q6" s="1"/>
+    </row>
+    <row r="7" spans="1:17">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -672,8 +687,9 @@
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
       <c r="P7" s="1"/>
-    </row>
-    <row r="8" spans="1:16">
+      <c r="Q7" s="1"/>
+    </row>
+    <row r="8" spans="1:17">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -690,8 +706,9 @@
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
-    </row>
-    <row r="9" spans="1:16">
+      <c r="Q8" s="1"/>
+    </row>
+    <row r="9" spans="1:17">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -708,8 +725,9 @@
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
       <c r="P9" s="1"/>
-    </row>
-    <row r="10" spans="1:16">
+      <c r="Q9" s="1"/>
+    </row>
+    <row r="10" spans="1:17">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -726,8 +744,9 @@
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
       <c r="P10" s="1"/>
-    </row>
-    <row r="11" spans="1:16">
+      <c r="Q10" s="1"/>
+    </row>
+    <row r="11" spans="1:17">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -744,8 +763,9 @@
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
       <c r="P11" s="1"/>
-    </row>
-    <row r="12" spans="1:16">
+      <c r="Q11" s="1"/>
+    </row>
+    <row r="12" spans="1:17">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -762,8 +782,9 @@
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
       <c r="P12" s="1"/>
-    </row>
-    <row r="13" spans="1:16">
+      <c r="Q12" s="1"/>
+    </row>
+    <row r="13" spans="1:17">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -780,8 +801,9 @@
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
       <c r="P13" s="1"/>
-    </row>
-    <row r="14" spans="1:16">
+      <c r="Q13" s="1"/>
+    </row>
+    <row r="14" spans="1:17">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -798,8 +820,9 @@
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
       <c r="P14" s="1"/>
-    </row>
-    <row r="15" spans="1:16">
+      <c r="Q14" s="1"/>
+    </row>
+    <row r="15" spans="1:17">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -816,8 +839,9 @@
       <c r="N15" s="1"/>
       <c r="O15" s="1"/>
       <c r="P15" s="1"/>
-    </row>
-    <row r="16" spans="1:16">
+      <c r="Q15" s="1"/>
+    </row>
+    <row r="16" spans="1:17">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -834,8 +858,9 @@
       <c r="N16" s="1"/>
       <c r="O16" s="1"/>
       <c r="P16" s="1"/>
-    </row>
-    <row r="17" spans="1:16">
+      <c r="Q16" s="1"/>
+    </row>
+    <row r="17" spans="1:17">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -852,8 +877,9 @@
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>
-    </row>
-    <row r="18" spans="1:16">
+      <c r="Q17" s="1"/>
+    </row>
+    <row r="18" spans="1:17">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -870,8 +896,9 @@
       <c r="N18" s="1"/>
       <c r="O18" s="1"/>
       <c r="P18" s="1"/>
-    </row>
-    <row r="19" spans="1:16">
+      <c r="Q18" s="1"/>
+    </row>
+    <row r="19" spans="1:17">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -888,8 +915,9 @@
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
       <c r="P19" s="1"/>
-    </row>
-    <row r="20" spans="1:16">
+      <c r="Q19" s="1"/>
+    </row>
+    <row r="20" spans="1:17">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -906,8 +934,9 @@
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
       <c r="P20" s="1"/>
-    </row>
-    <row r="21" spans="1:16">
+      <c r="Q20" s="1"/>
+    </row>
+    <row r="21" spans="1:17">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -924,8 +953,9 @@
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
       <c r="P21" s="1"/>
-    </row>
-    <row r="22" spans="1:16">
+      <c r="Q21" s="1"/>
+    </row>
+    <row r="22" spans="1:17">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -942,8 +972,9 @@
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
       <c r="P22" s="1"/>
-    </row>
-    <row r="23" spans="1:16">
+      <c r="Q22" s="1"/>
+    </row>
+    <row r="23" spans="1:17">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -960,8 +991,9 @@
       <c r="N23" s="1"/>
       <c r="O23" s="1"/>
       <c r="P23" s="1"/>
-    </row>
-    <row r="24" spans="1:16">
+      <c r="Q23" s="1"/>
+    </row>
+    <row r="24" spans="1:17">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -978,8 +1010,9 @@
       <c r="N24" s="1"/>
       <c r="O24" s="1"/>
       <c r="P24" s="1"/>
-    </row>
-    <row r="25" spans="1:16">
+      <c r="Q24" s="1"/>
+    </row>
+    <row r="25" spans="1:17">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -996,8 +1029,9 @@
       <c r="N25" s="1"/>
       <c r="O25" s="1"/>
       <c r="P25" s="1"/>
-    </row>
-    <row r="26" spans="1:16">
+      <c r="Q25" s="1"/>
+    </row>
+    <row r="26" spans="1:17">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1014,8 +1048,9 @@
       <c r="N26" s="1"/>
       <c r="O26" s="1"/>
       <c r="P26" s="1"/>
-    </row>
-    <row r="27" spans="1:16">
+      <c r="Q26" s="1"/>
+    </row>
+    <row r="27" spans="1:17">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -1032,8 +1067,9 @@
       <c r="N27" s="1"/>
       <c r="O27" s="1"/>
       <c r="P27" s="1"/>
-    </row>
-    <row r="28" spans="1:16">
+      <c r="Q27" s="1"/>
+    </row>
+    <row r="28" spans="1:17">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -1050,8 +1086,9 @@
       <c r="N28" s="1"/>
       <c r="O28" s="1"/>
       <c r="P28" s="1"/>
-    </row>
-    <row r="29" spans="1:16">
+      <c r="Q28" s="1"/>
+    </row>
+    <row r="29" spans="1:17">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -1068,8 +1105,9 @@
       <c r="N29" s="1"/>
       <c r="O29" s="1"/>
       <c r="P29" s="1"/>
-    </row>
-    <row r="30" spans="1:16">
+      <c r="Q29" s="1"/>
+    </row>
+    <row r="30" spans="1:17">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -1086,8 +1124,9 @@
       <c r="N30" s="1"/>
       <c r="O30" s="1"/>
       <c r="P30" s="1"/>
-    </row>
-    <row r="31" spans="1:16">
+      <c r="Q30" s="1"/>
+    </row>
+    <row r="31" spans="1:17">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -1104,8 +1143,9 @@
       <c r="N31" s="1"/>
       <c r="O31" s="1"/>
       <c r="P31" s="1"/>
-    </row>
-    <row r="32" spans="1:16">
+      <c r="Q31" s="1"/>
+    </row>
+    <row r="32" spans="1:17">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -1122,8 +1162,9 @@
       <c r="N32" s="1"/>
       <c r="O32" s="1"/>
       <c r="P32" s="1"/>
-    </row>
-    <row r="33" spans="1:16">
+      <c r="Q32" s="1"/>
+    </row>
+    <row r="33" spans="1:17">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -1140,8 +1181,9 @@
       <c r="N33" s="1"/>
       <c r="O33" s="1"/>
       <c r="P33" s="1"/>
-    </row>
-    <row r="34" spans="1:16">
+      <c r="Q33" s="1"/>
+    </row>
+    <row r="34" spans="1:17">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -1158,8 +1200,9 @@
       <c r="N34" s="1"/>
       <c r="O34" s="1"/>
       <c r="P34" s="1"/>
-    </row>
-    <row r="35" spans="1:16">
+      <c r="Q34" s="1"/>
+    </row>
+    <row r="35" spans="1:17">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -1176,8 +1219,9 @@
       <c r="N35" s="1"/>
       <c r="O35" s="1"/>
       <c r="P35" s="1"/>
-    </row>
-    <row r="36" spans="1:16">
+      <c r="Q35" s="1"/>
+    </row>
+    <row r="36" spans="1:17">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -1194,8 +1238,9 @@
       <c r="N36" s="1"/>
       <c r="O36" s="1"/>
       <c r="P36" s="1"/>
-    </row>
-    <row r="37" spans="1:16">
+      <c r="Q36" s="1"/>
+    </row>
+    <row r="37" spans="1:17">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -1212,8 +1257,9 @@
       <c r="N37" s="1"/>
       <c r="O37" s="1"/>
       <c r="P37" s="1"/>
-    </row>
-    <row r="38" spans="1:16">
+      <c r="Q37" s="1"/>
+    </row>
+    <row r="38" spans="1:17">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -1230,8 +1276,9 @@
       <c r="N38" s="1"/>
       <c r="O38" s="1"/>
       <c r="P38" s="1"/>
-    </row>
-    <row r="39" spans="1:16">
+      <c r="Q38" s="1"/>
+    </row>
+    <row r="39" spans="1:17">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -1248,8 +1295,9 @@
       <c r="N39" s="1"/>
       <c r="O39" s="1"/>
       <c r="P39" s="1"/>
-    </row>
-    <row r="40" spans="1:16">
+      <c r="Q39" s="1"/>
+    </row>
+    <row r="40" spans="1:17">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -1266,8 +1314,9 @@
       <c r="N40" s="1"/>
       <c r="O40" s="1"/>
       <c r="P40" s="1"/>
-    </row>
-    <row r="41" spans="1:16">
+      <c r="Q40" s="1"/>
+    </row>
+    <row r="41" spans="1:17">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -1284,8 +1333,9 @@
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
       <c r="P41" s="1"/>
-    </row>
-    <row r="42" spans="1:16">
+      <c r="Q41" s="1"/>
+    </row>
+    <row r="42" spans="1:17">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -1302,8 +1352,9 @@
       <c r="N42" s="1"/>
       <c r="O42" s="1"/>
       <c r="P42" s="1"/>
-    </row>
-    <row r="43" spans="1:16">
+      <c r="Q42" s="1"/>
+    </row>
+    <row r="43" spans="1:17">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -1320,8 +1371,9 @@
       <c r="N43" s="1"/>
       <c r="O43" s="1"/>
       <c r="P43" s="1"/>
-    </row>
-    <row r="44" spans="1:16">
+      <c r="Q43" s="1"/>
+    </row>
+    <row r="44" spans="1:17">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -1338,8 +1390,9 @@
       <c r="N44" s="1"/>
       <c r="O44" s="1"/>
       <c r="P44" s="1"/>
-    </row>
-    <row r="45" spans="1:16">
+      <c r="Q44" s="1"/>
+    </row>
+    <row r="45" spans="1:17">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -1356,8 +1409,9 @@
       <c r="N45" s="1"/>
       <c r="O45" s="1"/>
       <c r="P45" s="1"/>
-    </row>
-    <row r="46" spans="1:16">
+      <c r="Q45" s="1"/>
+    </row>
+    <row r="46" spans="1:17">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -1374,8 +1428,9 @@
       <c r="N46" s="1"/>
       <c r="O46" s="1"/>
       <c r="P46" s="1"/>
-    </row>
-    <row r="47" spans="1:16">
+      <c r="Q46" s="1"/>
+    </row>
+    <row r="47" spans="1:17">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -1392,8 +1447,9 @@
       <c r="N47" s="1"/>
       <c r="O47" s="1"/>
       <c r="P47" s="1"/>
-    </row>
-    <row r="48" spans="1:16">
+      <c r="Q47" s="1"/>
+    </row>
+    <row r="48" spans="1:17">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -1410,8 +1466,9 @@
       <c r="N48" s="1"/>
       <c r="O48" s="1"/>
       <c r="P48" s="1"/>
-    </row>
-    <row r="49" spans="1:16">
+      <c r="Q48" s="1"/>
+    </row>
+    <row r="49" spans="1:17">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -1428,8 +1485,9 @@
       <c r="N49" s="1"/>
       <c r="O49" s="1"/>
       <c r="P49" s="1"/>
-    </row>
-    <row r="50" spans="1:16">
+      <c r="Q49" s="1"/>
+    </row>
+    <row r="50" spans="1:17">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -1446,8 +1504,9 @@
       <c r="N50" s="1"/>
       <c r="O50" s="1"/>
       <c r="P50" s="1"/>
-    </row>
-    <row r="51" spans="1:16">
+      <c r="Q50" s="1"/>
+    </row>
+    <row r="51" spans="1:17">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
@@ -1464,8 +1523,9 @@
       <c r="N51" s="1"/>
       <c r="O51" s="1"/>
       <c r="P51" s="1"/>
-    </row>
-    <row r="52" spans="1:16">
+      <c r="Q51" s="1"/>
+    </row>
+    <row r="52" spans="1:17">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
@@ -1482,8 +1542,9 @@
       <c r="N52" s="1"/>
       <c r="O52" s="1"/>
       <c r="P52" s="1"/>
-    </row>
-    <row r="53" spans="1:16">
+      <c r="Q52" s="1"/>
+    </row>
+    <row r="53" spans="1:17">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -1500,8 +1561,9 @@
       <c r="N53" s="1"/>
       <c r="O53" s="1"/>
       <c r="P53" s="1"/>
-    </row>
-    <row r="54" spans="1:16">
+      <c r="Q53" s="1"/>
+    </row>
+    <row r="54" spans="1:17">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
@@ -1518,8 +1580,9 @@
       <c r="N54" s="1"/>
       <c r="O54" s="1"/>
       <c r="P54" s="1"/>
-    </row>
-    <row r="55" spans="1:16">
+      <c r="Q54" s="1"/>
+    </row>
+    <row r="55" spans="1:17">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -1536,8 +1599,9 @@
       <c r="N55" s="1"/>
       <c r="O55" s="1"/>
       <c r="P55" s="1"/>
-    </row>
-    <row r="56" spans="1:16">
+      <c r="Q55" s="1"/>
+    </row>
+    <row r="56" spans="1:17">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
@@ -1554,8 +1618,9 @@
       <c r="N56" s="1"/>
       <c r="O56" s="1"/>
       <c r="P56" s="1"/>
-    </row>
-    <row r="57" spans="1:16">
+      <c r="Q56" s="1"/>
+    </row>
+    <row r="57" spans="1:17">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
@@ -1572,8 +1637,9 @@
       <c r="N57" s="1"/>
       <c r="O57" s="1"/>
       <c r="P57" s="1"/>
-    </row>
-    <row r="58" spans="1:16">
+      <c r="Q57" s="1"/>
+    </row>
+    <row r="58" spans="1:17">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
@@ -1590,8 +1656,9 @@
       <c r="N58" s="1"/>
       <c r="O58" s="1"/>
       <c r="P58" s="1"/>
-    </row>
-    <row r="59" spans="1:16">
+      <c r="Q58" s="1"/>
+    </row>
+    <row r="59" spans="1:17">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
@@ -1608,8 +1675,9 @@
       <c r="N59" s="1"/>
       <c r="O59" s="1"/>
       <c r="P59" s="1"/>
-    </row>
-    <row r="60" spans="1:16">
+      <c r="Q59" s="1"/>
+    </row>
+    <row r="60" spans="1:17">
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
@@ -1626,8 +1694,9 @@
       <c r="N60" s="1"/>
       <c r="O60" s="1"/>
       <c r="P60" s="1"/>
-    </row>
-    <row r="61" spans="1:16">
+      <c r="Q60" s="1"/>
+    </row>
+    <row r="61" spans="1:17">
       <c r="A61" s="1"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
@@ -1644,8 +1713,9 @@
       <c r="N61" s="1"/>
       <c r="O61" s="1"/>
       <c r="P61" s="1"/>
-    </row>
-    <row r="62" spans="1:16">
+      <c r="Q61" s="1"/>
+    </row>
+    <row r="62" spans="1:17">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
@@ -1662,8 +1732,9 @@
       <c r="N62" s="1"/>
       <c r="O62" s="1"/>
       <c r="P62" s="1"/>
-    </row>
-    <row r="63" spans="1:16">
+      <c r="Q62" s="1"/>
+    </row>
+    <row r="63" spans="1:17">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
@@ -1680,8 +1751,9 @@
       <c r="N63" s="1"/>
       <c r="O63" s="1"/>
       <c r="P63" s="1"/>
-    </row>
-    <row r="64" spans="1:16">
+      <c r="Q63" s="1"/>
+    </row>
+    <row r="64" spans="1:17">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
@@ -1698,8 +1770,9 @@
       <c r="N64" s="1"/>
       <c r="O64" s="1"/>
       <c r="P64" s="1"/>
-    </row>
-    <row r="65" spans="1:16">
+      <c r="Q64" s="1"/>
+    </row>
+    <row r="65" spans="1:17">
       <c r="A65" s="1"/>
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
@@ -1716,8 +1789,9 @@
       <c r="N65" s="1"/>
       <c r="O65" s="1"/>
       <c r="P65" s="1"/>
-    </row>
-    <row r="66" spans="1:16">
+      <c r="Q65" s="1"/>
+    </row>
+    <row r="66" spans="1:17">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>
@@ -1734,8 +1808,9 @@
       <c r="N66" s="1"/>
       <c r="O66" s="1"/>
       <c r="P66" s="1"/>
-    </row>
-    <row r="67" spans="1:16">
+      <c r="Q66" s="1"/>
+    </row>
+    <row r="67" spans="1:17">
       <c r="A67" s="1"/>
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
@@ -1752,8 +1827,9 @@
       <c r="N67" s="1"/>
       <c r="O67" s="1"/>
       <c r="P67" s="1"/>
-    </row>
-    <row r="68" spans="1:16">
+      <c r="Q67" s="1"/>
+    </row>
+    <row r="68" spans="1:17">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
@@ -1770,8 +1846,9 @@
       <c r="N68" s="1"/>
       <c r="O68" s="1"/>
       <c r="P68" s="1"/>
-    </row>
-    <row r="69" spans="1:16">
+      <c r="Q68" s="1"/>
+    </row>
+    <row r="69" spans="1:17">
       <c r="A69" s="1"/>
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
@@ -1788,8 +1865,9 @@
       <c r="N69" s="1"/>
       <c r="O69" s="1"/>
       <c r="P69" s="1"/>
-    </row>
-    <row r="70" spans="1:16">
+      <c r="Q69" s="1"/>
+    </row>
+    <row r="70" spans="1:17">
       <c r="A70" s="1"/>
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
@@ -1806,8 +1884,9 @@
       <c r="N70" s="1"/>
       <c r="O70" s="1"/>
       <c r="P70" s="1"/>
-    </row>
-    <row r="71" spans="1:16">
+      <c r="Q70" s="1"/>
+    </row>
+    <row r="71" spans="1:17">
       <c r="A71" s="1"/>
       <c r="B71" s="1"/>
       <c r="C71" s="1"/>
@@ -1824,8 +1903,9 @@
       <c r="N71" s="1"/>
       <c r="O71" s="1"/>
       <c r="P71" s="1"/>
-    </row>
-    <row r="72" spans="1:16">
+      <c r="Q71" s="1"/>
+    </row>
+    <row r="72" spans="1:17">
       <c r="A72" s="1"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
@@ -1842,8 +1922,9 @@
       <c r="N72" s="1"/>
       <c r="O72" s="1"/>
       <c r="P72" s="1"/>
-    </row>
-    <row r="73" spans="1:16">
+      <c r="Q72" s="1"/>
+    </row>
+    <row r="73" spans="1:17">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
@@ -1860,8 +1941,9 @@
       <c r="N73" s="1"/>
       <c r="O73" s="1"/>
       <c r="P73" s="1"/>
-    </row>
-    <row r="74" spans="1:16">
+      <c r="Q73" s="1"/>
+    </row>
+    <row r="74" spans="1:17">
       <c r="A74" s="1"/>
       <c r="B74" s="1"/>
       <c r="C74" s="1"/>
@@ -1878,8 +1960,9 @@
       <c r="N74" s="1"/>
       <c r="O74" s="1"/>
       <c r="P74" s="1"/>
-    </row>
-    <row r="75" spans="1:16">
+      <c r="Q74" s="1"/>
+    </row>
+    <row r="75" spans="1:17">
       <c r="A75" s="1"/>
       <c r="B75" s="1"/>
       <c r="C75" s="1"/>
@@ -1896,8 +1979,9 @@
       <c r="N75" s="1"/>
       <c r="O75" s="1"/>
       <c r="P75" s="1"/>
-    </row>
-    <row r="76" spans="1:16">
+      <c r="Q75" s="1"/>
+    </row>
+    <row r="76" spans="1:17">
       <c r="A76" s="1"/>
       <c r="B76" s="1"/>
       <c r="C76" s="1"/>
@@ -1914,8 +1998,9 @@
       <c r="N76" s="1"/>
       <c r="O76" s="1"/>
       <c r="P76" s="1"/>
-    </row>
-    <row r="77" spans="1:16">
+      <c r="Q76" s="1"/>
+    </row>
+    <row r="77" spans="1:17">
       <c r="A77" s="1"/>
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
@@ -1932,8 +2017,9 @@
       <c r="N77" s="1"/>
       <c r="O77" s="1"/>
       <c r="P77" s="1"/>
-    </row>
-    <row r="78" spans="1:16">
+      <c r="Q77" s="1"/>
+    </row>
+    <row r="78" spans="1:17">
       <c r="A78" s="1"/>
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
@@ -1950,8 +2036,9 @@
       <c r="N78" s="1"/>
       <c r="O78" s="1"/>
       <c r="P78" s="1"/>
-    </row>
-    <row r="79" spans="1:16">
+      <c r="Q78" s="1"/>
+    </row>
+    <row r="79" spans="1:17">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
@@ -1968,8 +2055,9 @@
       <c r="N79" s="1"/>
       <c r="O79" s="1"/>
       <c r="P79" s="1"/>
-    </row>
-    <row r="80" spans="1:16">
+      <c r="Q79" s="1"/>
+    </row>
+    <row r="80" spans="1:17">
       <c r="A80" s="1"/>
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
@@ -1986,8 +2074,9 @@
       <c r="N80" s="1"/>
       <c r="O80" s="1"/>
       <c r="P80" s="1"/>
-    </row>
-    <row r="81" spans="1:16">
+      <c r="Q80" s="1"/>
+    </row>
+    <row r="81" spans="1:17">
       <c r="A81" s="1"/>
       <c r="B81" s="1"/>
       <c r="C81" s="1"/>
@@ -2004,8 +2093,9 @@
       <c r="N81" s="1"/>
       <c r="O81" s="1"/>
       <c r="P81" s="1"/>
-    </row>
-    <row r="82" spans="1:16">
+      <c r="Q81" s="1"/>
+    </row>
+    <row r="82" spans="1:17">
       <c r="A82" s="1"/>
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
@@ -2022,8 +2112,9 @@
       <c r="N82" s="1"/>
       <c r="O82" s="1"/>
       <c r="P82" s="1"/>
-    </row>
-    <row r="83" spans="1:16">
+      <c r="Q82" s="1"/>
+    </row>
+    <row r="83" spans="1:17">
       <c r="A83" s="1"/>
       <c r="B83" s="1"/>
       <c r="C83" s="1"/>
@@ -2040,8 +2131,9 @@
       <c r="N83" s="1"/>
       <c r="O83" s="1"/>
       <c r="P83" s="1"/>
-    </row>
-    <row r="84" spans="1:16">
+      <c r="Q83" s="1"/>
+    </row>
+    <row r="84" spans="1:17">
       <c r="A84" s="1"/>
       <c r="B84" s="1"/>
       <c r="C84" s="1"/>
@@ -2058,8 +2150,9 @@
       <c r="N84" s="1"/>
       <c r="O84" s="1"/>
       <c r="P84" s="1"/>
-    </row>
-    <row r="85" spans="1:16">
+      <c r="Q84" s="1"/>
+    </row>
+    <row r="85" spans="1:17">
       <c r="A85" s="1"/>
       <c r="B85" s="1"/>
       <c r="C85" s="1"/>
@@ -2076,8 +2169,9 @@
       <c r="N85" s="1"/>
       <c r="O85" s="1"/>
       <c r="P85" s="1"/>
-    </row>
-    <row r="86" spans="1:16">
+      <c r="Q85" s="1"/>
+    </row>
+    <row r="86" spans="1:17">
       <c r="A86" s="1"/>
       <c r="B86" s="1"/>
       <c r="C86" s="1"/>
@@ -2094,8 +2188,9 @@
       <c r="N86" s="1"/>
       <c r="O86" s="1"/>
       <c r="P86" s="1"/>
-    </row>
-    <row r="87" spans="1:16">
+      <c r="Q86" s="1"/>
+    </row>
+    <row r="87" spans="1:17">
       <c r="A87" s="1"/>
       <c r="B87" s="1"/>
       <c r="C87" s="1"/>
@@ -2112,8 +2207,9 @@
       <c r="N87" s="1"/>
       <c r="O87" s="1"/>
       <c r="P87" s="1"/>
-    </row>
-    <row r="88" spans="1:16">
+      <c r="Q87" s="1"/>
+    </row>
+    <row r="88" spans="1:17">
       <c r="A88" s="1"/>
       <c r="B88" s="1"/>
       <c r="C88" s="1"/>
@@ -2130,8 +2226,9 @@
       <c r="N88" s="1"/>
       <c r="O88" s="1"/>
       <c r="P88" s="1"/>
-    </row>
-    <row r="89" spans="1:16">
+      <c r="Q88" s="1"/>
+    </row>
+    <row r="89" spans="1:17">
       <c r="A89" s="1"/>
       <c r="B89" s="1"/>
       <c r="C89" s="1"/>
@@ -2148,8 +2245,9 @@
       <c r="N89" s="1"/>
       <c r="O89" s="1"/>
       <c r="P89" s="1"/>
-    </row>
-    <row r="90" spans="1:16">
+      <c r="Q89" s="1"/>
+    </row>
+    <row r="90" spans="1:17">
       <c r="A90" s="1"/>
       <c r="B90" s="1"/>
       <c r="C90" s="1"/>
@@ -2166,8 +2264,9 @@
       <c r="N90" s="1"/>
       <c r="O90" s="1"/>
       <c r="P90" s="1"/>
-    </row>
-    <row r="91" spans="1:16">
+      <c r="Q90" s="1"/>
+    </row>
+    <row r="91" spans="1:17">
       <c r="A91" s="1"/>
       <c r="B91" s="1"/>
       <c r="C91" s="1"/>
@@ -2184,8 +2283,9 @@
       <c r="N91" s="1"/>
       <c r="O91" s="1"/>
       <c r="P91" s="1"/>
-    </row>
-    <row r="92" spans="1:16">
+      <c r="Q91" s="1"/>
+    </row>
+    <row r="92" spans="1:17">
       <c r="A92" s="1"/>
       <c r="B92" s="1"/>
       <c r="C92" s="1"/>
@@ -2202,8 +2302,9 @@
       <c r="N92" s="1"/>
       <c r="O92" s="1"/>
       <c r="P92" s="1"/>
-    </row>
-    <row r="93" spans="1:16">
+      <c r="Q92" s="1"/>
+    </row>
+    <row r="93" spans="1:17">
       <c r="A93" s="1"/>
       <c r="B93" s="1"/>
       <c r="C93" s="1"/>
@@ -2220,8 +2321,9 @@
       <c r="N93" s="1"/>
       <c r="O93" s="1"/>
       <c r="P93" s="1"/>
-    </row>
-    <row r="94" spans="1:16">
+      <c r="Q93" s="1"/>
+    </row>
+    <row r="94" spans="1:17">
       <c r="A94" s="1"/>
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
@@ -2238,8 +2340,9 @@
       <c r="N94" s="1"/>
       <c r="O94" s="1"/>
       <c r="P94" s="1"/>
-    </row>
-    <row r="95" spans="1:16">
+      <c r="Q94" s="1"/>
+    </row>
+    <row r="95" spans="1:17">
       <c r="A95" s="1"/>
       <c r="B95" s="1"/>
       <c r="C95" s="1"/>
@@ -2256,8 +2359,9 @@
       <c r="N95" s="1"/>
       <c r="O95" s="1"/>
       <c r="P95" s="1"/>
-    </row>
-    <row r="96" spans="1:16">
+      <c r="Q95" s="1"/>
+    </row>
+    <row r="96" spans="1:17">
       <c r="A96" s="1"/>
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
@@ -2274,8 +2378,9 @@
       <c r="N96" s="1"/>
       <c r="O96" s="1"/>
       <c r="P96" s="1"/>
-    </row>
-    <row r="97" spans="1:16">
+      <c r="Q96" s="1"/>
+    </row>
+    <row r="97" spans="1:17">
       <c r="A97" s="1"/>
       <c r="B97" s="1"/>
       <c r="C97" s="1"/>
@@ -2292,8 +2397,9 @@
       <c r="N97" s="1"/>
       <c r="O97" s="1"/>
       <c r="P97" s="1"/>
-    </row>
-    <row r="98" spans="1:16">
+      <c r="Q97" s="1"/>
+    </row>
+    <row r="98" spans="1:17">
       <c r="A98" s="1"/>
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
@@ -2310,8 +2416,9 @@
       <c r="N98" s="1"/>
       <c r="O98" s="1"/>
       <c r="P98" s="1"/>
-    </row>
-    <row r="99" spans="1:16">
+      <c r="Q98" s="1"/>
+    </row>
+    <row r="99" spans="1:17">
       <c r="A99" s="1"/>
       <c r="B99" s="1"/>
       <c r="C99" s="1"/>
@@ -2328,8 +2435,9 @@
       <c r="N99" s="1"/>
       <c r="O99" s="1"/>
       <c r="P99" s="1"/>
-    </row>
-    <row r="100" spans="1:16">
+      <c r="Q99" s="1"/>
+    </row>
+    <row r="100" spans="1:17">
       <c r="A100" s="1"/>
       <c r="B100" s="1"/>
       <c r="C100" s="1"/>
@@ -2346,8 +2454,9 @@
       <c r="N100" s="1"/>
       <c r="O100" s="1"/>
       <c r="P100" s="1"/>
-    </row>
-    <row r="101" spans="1:16">
+      <c r="Q100" s="1"/>
+    </row>
+    <row r="101" spans="1:17">
       <c r="A101" s="1"/>
       <c r="B101" s="1"/>
       <c r="C101" s="1"/>
@@ -2364,8 +2473,9 @@
       <c r="N101" s="1"/>
       <c r="O101" s="1"/>
       <c r="P101" s="1"/>
-    </row>
-    <row r="102" spans="1:16">
+      <c r="Q101" s="1"/>
+    </row>
+    <row r="102" spans="1:17">
       <c r="A102" s="1"/>
       <c r="B102" s="1"/>
       <c r="C102" s="1"/>
@@ -2382,8 +2492,9 @@
       <c r="N102" s="1"/>
       <c r="O102" s="1"/>
       <c r="P102" s="1"/>
-    </row>
-    <row r="103" spans="1:16">
+      <c r="Q102" s="1"/>
+    </row>
+    <row r="103" spans="1:17">
       <c r="A103" s="1"/>
       <c r="B103" s="1"/>
       <c r="C103" s="1"/>
@@ -2400,8 +2511,9 @@
       <c r="N103" s="1"/>
       <c r="O103" s="1"/>
       <c r="P103" s="1"/>
-    </row>
-    <row r="104" spans="1:16">
+      <c r="Q103" s="1"/>
+    </row>
+    <row r="104" spans="1:17">
       <c r="A104" s="1"/>
       <c r="B104" s="1"/>
       <c r="C104" s="1"/>
@@ -2418,8 +2530,9 @@
       <c r="N104" s="1"/>
       <c r="O104" s="1"/>
       <c r="P104" s="1"/>
-    </row>
-    <row r="105" spans="1:16">
+      <c r="Q104" s="1"/>
+    </row>
+    <row r="105" spans="1:17">
       <c r="A105" s="1"/>
       <c r="B105" s="1"/>
       <c r="C105" s="1"/>
@@ -2436,8 +2549,9 @@
       <c r="N105" s="1"/>
       <c r="O105" s="1"/>
       <c r="P105" s="1"/>
-    </row>
-    <row r="106" spans="1:16">
+      <c r="Q105" s="1"/>
+    </row>
+    <row r="106" spans="1:17">
       <c r="A106" s="1"/>
       <c r="B106" s="1"/>
       <c r="C106" s="1"/>
@@ -2454,8 +2568,9 @@
       <c r="N106" s="1"/>
       <c r="O106" s="1"/>
       <c r="P106" s="1"/>
-    </row>
-    <row r="107" spans="1:16">
+      <c r="Q106" s="1"/>
+    </row>
+    <row r="107" spans="1:17">
       <c r="A107" s="1"/>
       <c r="B107" s="1"/>
       <c r="C107" s="1"/>
@@ -2472,8 +2587,9 @@
       <c r="N107" s="1"/>
       <c r="O107" s="1"/>
       <c r="P107" s="1"/>
-    </row>
-    <row r="108" spans="1:16">
+      <c r="Q107" s="1"/>
+    </row>
+    <row r="108" spans="1:17">
       <c r="A108" s="1"/>
       <c r="B108" s="1"/>
       <c r="C108" s="1"/>
@@ -2490,8 +2606,9 @@
       <c r="N108" s="1"/>
       <c r="O108" s="1"/>
       <c r="P108" s="1"/>
-    </row>
-    <row r="109" spans="1:16">
+      <c r="Q108" s="1"/>
+    </row>
+    <row r="109" spans="1:17">
       <c r="A109" s="1"/>
       <c r="B109" s="1"/>
       <c r="C109" s="1"/>
@@ -2508,8 +2625,9 @@
       <c r="N109" s="1"/>
       <c r="O109" s="1"/>
       <c r="P109" s="1"/>
-    </row>
-    <row r="110" spans="1:16">
+      <c r="Q109" s="1"/>
+    </row>
+    <row r="110" spans="1:17">
       <c r="A110" s="1"/>
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
@@ -2526,8 +2644,9 @@
       <c r="N110" s="1"/>
       <c r="O110" s="1"/>
       <c r="P110" s="1"/>
-    </row>
-    <row r="111" spans="1:16">
+      <c r="Q110" s="1"/>
+    </row>
+    <row r="111" spans="1:17">
       <c r="A111" s="1"/>
       <c r="B111" s="1"/>
       <c r="C111" s="1"/>
@@ -2544,8 +2663,9 @@
       <c r="N111" s="1"/>
       <c r="O111" s="1"/>
       <c r="P111" s="1"/>
-    </row>
-    <row r="112" spans="1:16">
+      <c r="Q111" s="1"/>
+    </row>
+    <row r="112" spans="1:17">
       <c r="A112" s="1"/>
       <c r="B112" s="1"/>
       <c r="C112" s="1"/>
@@ -2562,8 +2682,9 @@
       <c r="N112" s="1"/>
       <c r="O112" s="1"/>
       <c r="P112" s="1"/>
-    </row>
-    <row r="113" spans="1:16">
+      <c r="Q112" s="1"/>
+    </row>
+    <row r="113" spans="1:17">
       <c r="A113" s="1"/>
       <c r="B113" s="1"/>
       <c r="C113" s="1"/>
@@ -2580,8 +2701,9 @@
       <c r="N113" s="1"/>
       <c r="O113" s="1"/>
       <c r="P113" s="1"/>
-    </row>
-    <row r="114" spans="1:16">
+      <c r="Q113" s="1"/>
+    </row>
+    <row r="114" spans="1:17">
       <c r="A114" s="1"/>
       <c r="B114" s="1"/>
       <c r="C114" s="1"/>
@@ -2598,8 +2720,9 @@
       <c r="N114" s="1"/>
       <c r="O114" s="1"/>
       <c r="P114" s="1"/>
-    </row>
-    <row r="115" spans="1:16">
+      <c r="Q114" s="1"/>
+    </row>
+    <row r="115" spans="1:17">
       <c r="A115" s="1"/>
       <c r="B115" s="1"/>
       <c r="C115" s="1"/>
@@ -2616,8 +2739,9 @@
       <c r="N115" s="1"/>
       <c r="O115" s="1"/>
       <c r="P115" s="1"/>
-    </row>
-    <row r="116" spans="1:16">
+      <c r="Q115" s="1"/>
+    </row>
+    <row r="116" spans="1:17">
       <c r="A116" s="1"/>
       <c r="B116" s="1"/>
       <c r="C116" s="1"/>
@@ -2634,8 +2758,9 @@
       <c r="N116" s="1"/>
       <c r="O116" s="1"/>
       <c r="P116" s="1"/>
-    </row>
-    <row r="117" spans="1:16">
+      <c r="Q116" s="1"/>
+    </row>
+    <row r="117" spans="1:17">
       <c r="A117" s="1"/>
       <c r="B117" s="1"/>
       <c r="C117" s="1"/>
@@ -2652,8 +2777,9 @@
       <c r="N117" s="1"/>
       <c r="O117" s="1"/>
       <c r="P117" s="1"/>
-    </row>
-    <row r="118" spans="1:16">
+      <c r="Q117" s="1"/>
+    </row>
+    <row r="118" spans="1:17">
       <c r="A118" s="1"/>
       <c r="B118" s="1"/>
       <c r="C118" s="1"/>
@@ -2670,8 +2796,9 @@
       <c r="N118" s="1"/>
       <c r="O118" s="1"/>
       <c r="P118" s="1"/>
-    </row>
-    <row r="119" spans="1:16">
+      <c r="Q118" s="1"/>
+    </row>
+    <row r="119" spans="1:17">
       <c r="A119" s="1"/>
       <c r="B119" s="1"/>
       <c r="C119" s="1"/>
@@ -2688,8 +2815,9 @@
       <c r="N119" s="1"/>
       <c r="O119" s="1"/>
       <c r="P119" s="1"/>
-    </row>
-    <row r="120" spans="1:16">
+      <c r="Q119" s="1"/>
+    </row>
+    <row r="120" spans="1:17">
       <c r="A120" s="1"/>
       <c r="B120" s="1"/>
       <c r="C120" s="1"/>
@@ -2706,8 +2834,9 @@
       <c r="N120" s="1"/>
       <c r="O120" s="1"/>
       <c r="P120" s="1"/>
-    </row>
-    <row r="121" spans="1:16">
+      <c r="Q120" s="1"/>
+    </row>
+    <row r="121" spans="1:17">
       <c r="A121" s="1"/>
       <c r="B121" s="1"/>
       <c r="C121" s="1"/>
@@ -2724,8 +2853,9 @@
       <c r="N121" s="1"/>
       <c r="O121" s="1"/>
       <c r="P121" s="1"/>
-    </row>
-    <row r="122" spans="1:16">
+      <c r="Q121" s="1"/>
+    </row>
+    <row r="122" spans="1:17">
       <c r="A122" s="1"/>
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
@@ -2742,8 +2872,9 @@
       <c r="N122" s="1"/>
       <c r="O122" s="1"/>
       <c r="P122" s="1"/>
-    </row>
-    <row r="123" spans="1:16">
+      <c r="Q122" s="1"/>
+    </row>
+    <row r="123" spans="1:17">
       <c r="A123" s="1"/>
       <c r="B123" s="1"/>
       <c r="C123" s="1"/>
@@ -2760,8 +2891,9 @@
       <c r="N123" s="1"/>
       <c r="O123" s="1"/>
       <c r="P123" s="1"/>
-    </row>
-    <row r="124" spans="1:16">
+      <c r="Q123" s="1"/>
+    </row>
+    <row r="124" spans="1:17">
       <c r="A124" s="1"/>
       <c r="B124" s="1"/>
       <c r="C124" s="1"/>
@@ -2778,8 +2910,9 @@
       <c r="N124" s="1"/>
       <c r="O124" s="1"/>
       <c r="P124" s="1"/>
-    </row>
-    <row r="125" spans="1:16">
+      <c r="Q124" s="1"/>
+    </row>
+    <row r="125" spans="1:17">
       <c r="A125" s="1"/>
       <c r="B125" s="1"/>
       <c r="C125" s="1"/>
@@ -2796,8 +2929,9 @@
       <c r="N125" s="1"/>
       <c r="O125" s="1"/>
       <c r="P125" s="1"/>
-    </row>
-    <row r="126" spans="1:16">
+      <c r="Q125" s="1"/>
+    </row>
+    <row r="126" spans="1:17">
       <c r="A126" s="1"/>
       <c r="B126" s="1"/>
       <c r="C126" s="1"/>
@@ -2814,8 +2948,9 @@
       <c r="N126" s="1"/>
       <c r="O126" s="1"/>
       <c r="P126" s="1"/>
-    </row>
-    <row r="127" spans="1:16">
+      <c r="Q126" s="1"/>
+    </row>
+    <row r="127" spans="1:17">
       <c r="A127" s="1"/>
       <c r="B127" s="1"/>
       <c r="C127" s="1"/>
@@ -2832,8 +2967,9 @@
       <c r="N127" s="1"/>
       <c r="O127" s="1"/>
       <c r="P127" s="1"/>
-    </row>
-    <row r="128" spans="1:16">
+      <c r="Q127" s="1"/>
+    </row>
+    <row r="128" spans="1:17">
       <c r="A128" s="1"/>
       <c r="B128" s="1"/>
       <c r="C128" s="1"/>
@@ -2850,8 +2986,9 @@
       <c r="N128" s="1"/>
       <c r="O128" s="1"/>
       <c r="P128" s="1"/>
-    </row>
-    <row r="129" spans="1:16">
+      <c r="Q128" s="1"/>
+    </row>
+    <row r="129" spans="1:17">
       <c r="A129" s="1"/>
       <c r="B129" s="1"/>
       <c r="C129" s="1"/>
@@ -2868,8 +3005,9 @@
       <c r="N129" s="1"/>
       <c r="O129" s="1"/>
       <c r="P129" s="1"/>
-    </row>
-    <row r="130" spans="1:16">
+      <c r="Q129" s="1"/>
+    </row>
+    <row r="130" spans="1:17">
       <c r="A130" s="1"/>
       <c r="B130" s="1"/>
       <c r="C130" s="1"/>
@@ -2886,8 +3024,9 @@
       <c r="N130" s="1"/>
       <c r="O130" s="1"/>
       <c r="P130" s="1"/>
-    </row>
-    <row r="131" spans="1:16">
+      <c r="Q130" s="1"/>
+    </row>
+    <row r="131" spans="1:17">
       <c r="A131" s="1"/>
       <c r="B131" s="1"/>
       <c r="C131" s="1"/>
@@ -2904,8 +3043,9 @@
       <c r="N131" s="1"/>
       <c r="O131" s="1"/>
       <c r="P131" s="1"/>
-    </row>
-    <row r="132" spans="1:16">
+      <c r="Q131" s="1"/>
+    </row>
+    <row r="132" spans="1:17">
       <c r="A132" s="1"/>
       <c r="B132" s="1"/>
       <c r="C132" s="1"/>
@@ -2922,8 +3062,9 @@
       <c r="N132" s="1"/>
       <c r="O132" s="1"/>
       <c r="P132" s="1"/>
-    </row>
-    <row r="133" spans="1:16">
+      <c r="Q132" s="1"/>
+    </row>
+    <row r="133" spans="1:17">
       <c r="A133" s="1"/>
       <c r="B133" s="1"/>
       <c r="C133" s="1"/>
@@ -2940,8 +3081,9 @@
       <c r="N133" s="1"/>
       <c r="O133" s="1"/>
       <c r="P133" s="1"/>
-    </row>
-    <row r="134" spans="1:16">
+      <c r="Q133" s="1"/>
+    </row>
+    <row r="134" spans="1:17">
       <c r="A134" s="1"/>
       <c r="B134" s="1"/>
       <c r="C134" s="1"/>
@@ -2958,8 +3100,9 @@
       <c r="N134" s="1"/>
       <c r="O134" s="1"/>
       <c r="P134" s="1"/>
-    </row>
-    <row r="135" spans="1:16">
+      <c r="Q134" s="1"/>
+    </row>
+    <row r="135" spans="1:17">
       <c r="A135" s="1"/>
       <c r="B135" s="1"/>
       <c r="C135" s="1"/>
@@ -2976,8 +3119,9 @@
       <c r="N135" s="1"/>
       <c r="O135" s="1"/>
       <c r="P135" s="1"/>
-    </row>
-    <row r="136" spans="1:16">
+      <c r="Q135" s="1"/>
+    </row>
+    <row r="136" spans="1:17">
       <c r="A136" s="1"/>
       <c r="B136" s="1"/>
       <c r="C136" s="1"/>
@@ -2994,8 +3138,9 @@
       <c r="N136" s="1"/>
       <c r="O136" s="1"/>
       <c r="P136" s="1"/>
-    </row>
-    <row r="137" spans="1:16">
+      <c r="Q136" s="1"/>
+    </row>
+    <row r="137" spans="1:17">
       <c r="A137" s="1"/>
       <c r="B137" s="1"/>
       <c r="C137" s="1"/>
@@ -3012,8 +3157,9 @@
       <c r="N137" s="1"/>
       <c r="O137" s="1"/>
       <c r="P137" s="1"/>
-    </row>
-    <row r="138" spans="1:16">
+      <c r="Q137" s="1"/>
+    </row>
+    <row r="138" spans="1:17">
       <c r="A138" s="1"/>
       <c r="B138" s="1"/>
       <c r="C138" s="1"/>
@@ -3030,8 +3176,9 @@
       <c r="N138" s="1"/>
       <c r="O138" s="1"/>
       <c r="P138" s="1"/>
-    </row>
-    <row r="139" spans="1:16">
+      <c r="Q138" s="1"/>
+    </row>
+    <row r="139" spans="1:17">
       <c r="A139" s="1"/>
       <c r="B139" s="1"/>
       <c r="C139" s="1"/>
@@ -3048,8 +3195,9 @@
       <c r="N139" s="1"/>
       <c r="O139" s="1"/>
       <c r="P139" s="1"/>
-    </row>
-    <row r="140" spans="1:16">
+      <c r="Q139" s="1"/>
+    </row>
+    <row r="140" spans="1:17">
       <c r="A140" s="1"/>
       <c r="B140" s="1"/>
       <c r="C140" s="1"/>
@@ -3066,8 +3214,9 @@
       <c r="N140" s="1"/>
       <c r="O140" s="1"/>
       <c r="P140" s="1"/>
-    </row>
-    <row r="141" spans="1:16">
+      <c r="Q140" s="1"/>
+    </row>
+    <row r="141" spans="1:17">
       <c r="A141" s="1"/>
       <c r="B141" s="1"/>
       <c r="C141" s="1"/>
@@ -3084,8 +3233,9 @@
       <c r="N141" s="1"/>
       <c r="O141" s="1"/>
       <c r="P141" s="1"/>
-    </row>
-    <row r="142" spans="1:16">
+      <c r="Q141" s="1"/>
+    </row>
+    <row r="142" spans="1:17">
       <c r="A142" s="1"/>
       <c r="B142" s="1"/>
       <c r="C142" s="1"/>
@@ -3102,8 +3252,9 @@
       <c r="N142" s="1"/>
       <c r="O142" s="1"/>
       <c r="P142" s="1"/>
-    </row>
-    <row r="143" spans="1:16">
+      <c r="Q142" s="1"/>
+    </row>
+    <row r="143" spans="1:17">
       <c r="A143" s="1"/>
       <c r="B143" s="1"/>
       <c r="C143" s="1"/>
@@ -3120,8 +3271,9 @@
       <c r="N143" s="1"/>
       <c r="O143" s="1"/>
       <c r="P143" s="1"/>
-    </row>
-    <row r="144" spans="1:16">
+      <c r="Q143" s="1"/>
+    </row>
+    <row r="144" spans="1:17">
       <c r="A144" s="1"/>
       <c r="B144" s="1"/>
       <c r="C144" s="1"/>
@@ -3138,8 +3290,9 @@
       <c r="N144" s="1"/>
       <c r="O144" s="1"/>
       <c r="P144" s="1"/>
-    </row>
-    <row r="145" spans="1:16">
+      <c r="Q144" s="1"/>
+    </row>
+    <row r="145" spans="1:17">
       <c r="A145" s="1"/>
       <c r="B145" s="1"/>
       <c r="C145" s="1"/>
@@ -3156,8 +3309,9 @@
       <c r="N145" s="1"/>
       <c r="O145" s="1"/>
       <c r="P145" s="1"/>
-    </row>
-    <row r="146" spans="1:16">
+      <c r="Q145" s="1"/>
+    </row>
+    <row r="146" spans="1:17">
       <c r="A146" s="1"/>
       <c r="B146" s="1"/>
       <c r="C146" s="1"/>
@@ -3174,8 +3328,9 @@
       <c r="N146" s="1"/>
       <c r="O146" s="1"/>
       <c r="P146" s="1"/>
-    </row>
-    <row r="147" spans="1:16">
+      <c r="Q146" s="1"/>
+    </row>
+    <row r="147" spans="1:17">
       <c r="A147" s="1"/>
       <c r="B147" s="1"/>
       <c r="C147" s="1"/>
@@ -3192,8 +3347,9 @@
       <c r="N147" s="1"/>
       <c r="O147" s="1"/>
       <c r="P147" s="1"/>
-    </row>
-    <row r="148" spans="1:16">
+      <c r="Q147" s="1"/>
+    </row>
+    <row r="148" spans="1:17">
       <c r="A148" s="1"/>
       <c r="B148" s="1"/>
       <c r="C148" s="1"/>
@@ -3210,8 +3366,9 @@
       <c r="N148" s="1"/>
       <c r="O148" s="1"/>
       <c r="P148" s="1"/>
-    </row>
-    <row r="149" spans="1:16">
+      <c r="Q148" s="1"/>
+    </row>
+    <row r="149" spans="1:17">
       <c r="A149" s="1"/>
       <c r="B149" s="1"/>
       <c r="C149" s="1"/>
@@ -3228,8 +3385,9 @@
       <c r="N149" s="1"/>
       <c r="O149" s="1"/>
       <c r="P149" s="1"/>
-    </row>
-    <row r="150" spans="1:16">
+      <c r="Q149" s="1"/>
+    </row>
+    <row r="150" spans="1:17">
       <c r="A150" s="1"/>
       <c r="B150" s="1"/>
       <c r="C150" s="1"/>
@@ -3246,8 +3404,9 @@
       <c r="N150" s="1"/>
       <c r="O150" s="1"/>
       <c r="P150" s="1"/>
-    </row>
-    <row r="151" spans="1:16">
+      <c r="Q150" s="1"/>
+    </row>
+    <row r="151" spans="1:17">
       <c r="A151" s="1"/>
       <c r="B151" s="1"/>
       <c r="C151" s="1"/>
@@ -3264,8 +3423,9 @@
       <c r="N151" s="1"/>
       <c r="O151" s="1"/>
       <c r="P151" s="1"/>
-    </row>
-    <row r="152" spans="1:16">
+      <c r="Q151" s="1"/>
+    </row>
+    <row r="152" spans="1:17">
       <c r="A152" s="1"/>
       <c r="B152" s="1"/>
       <c r="C152" s="1"/>
@@ -3282,8 +3442,9 @@
       <c r="N152" s="1"/>
       <c r="O152" s="1"/>
       <c r="P152" s="1"/>
-    </row>
-    <row r="153" spans="1:16">
+      <c r="Q152" s="1"/>
+    </row>
+    <row r="153" spans="1:17">
       <c r="A153" s="1"/>
       <c r="B153" s="1"/>
       <c r="C153" s="1"/>
@@ -3300,8 +3461,9 @@
       <c r="N153" s="1"/>
       <c r="O153" s="1"/>
       <c r="P153" s="1"/>
-    </row>
-    <row r="154" spans="1:16">
+      <c r="Q153" s="1"/>
+    </row>
+    <row r="154" spans="1:17">
       <c r="A154" s="1"/>
       <c r="B154" s="1"/>
       <c r="C154" s="1"/>
@@ -3318,6 +3480,7 @@
       <c r="N154" s="1"/>
       <c r="O154" s="1"/>
       <c r="P154" s="1"/>
+      <c r="Q154" s="1"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>

<commit_message>
Ship Skolaris employee load template, faculty memo absents, and HR email setup fixes.
Stream daily-loads for load templates with cache and streaming downloads; count faculty memo violations from teaching schedules without shift setup; widen HR setup email field and add Skolaris reference pull helpers.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/resources/templates/employee_salary_upload_template.xlsx
+++ b/resources/templates/employee_salary_upload_template.xlsx
@@ -2832,7 +2832,9 @@
       <c r="G7" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H7" s="1"/>
+      <c r="H7" s="1" t="s">
+        <v>40</v>
+      </c>
       <c r="I7" s="1" t="s">
         <v>41</v>
       </c>

</xml_diff>

<commit_message>
Log People360 1.0.27 and refresh employee upload templates.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/resources/templates/employee_salary_upload_template.xlsx
+++ b/resources/templates/employee_salary_upload_template.xlsx
@@ -2992,114 +2992,152 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:Q500"/>
+  <dimension ref="A1:Q479"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="9.10" style="1"/>
+    <col min="2" max="2" width="9.10" style="1"/>
+    <col min="3" max="3" width="9.10" style="1"/>
+    <col min="4" max="4" width="9.10" style="1"/>
+    <col min="5" max="5" width="9.10" style="1"/>
+    <col min="6" max="6" width="9.10" style="1"/>
+    <col min="7" max="7" width="9.10" style="1"/>
+    <col min="8" max="8" width="9.10" style="1"/>
+    <col min="9" max="9" width="9.10" style="1"/>
+    <col min="10" max="10" width="9.10" style="1"/>
+    <col min="11" max="11" width="9.10" style="1"/>
+    <col min="12" max="12" width="9.10" style="1"/>
+    <col min="13" max="13" width="9.10" style="1"/>
+    <col min="14" max="14" width="9.10" style="1"/>
+    <col min="15" max="15" width="9.10" style="1"/>
+    <col min="16" max="16" width="9.10" style="1"/>
+    <col min="17" max="17" width="9.10" style="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:17">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="P2" t="s">
+      <c r="P2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Q2" s="1" t="s">
         <v>33</v>
       </c>
+    </row>
+    <row r="3" spans="1:17">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="1"/>
     </row>
     <row r="4" spans="1:17">
       <c r="A4" s="1" t="s">
@@ -24469,405 +24507,6 @@
       <c r="P479" s="1"/>
       <c r="Q479" s="1"/>
     </row>
-    <row r="480" spans="1:17">
-      <c r="A480" s="1"/>
-      <c r="B480" s="1"/>
-      <c r="C480" s="1"/>
-      <c r="D480" s="1"/>
-      <c r="E480" s="1"/>
-      <c r="F480" s="1"/>
-      <c r="G480" s="1"/>
-      <c r="H480" s="1"/>
-      <c r="I480" s="1"/>
-      <c r="J480" s="1"/>
-      <c r="K480" s="1"/>
-      <c r="L480" s="1"/>
-      <c r="M480" s="1"/>
-      <c r="N480" s="1"/>
-      <c r="O480" s="1"/>
-      <c r="P480" s="1"/>
-      <c r="Q480" s="1"/>
-    </row>
-    <row r="481" spans="1:17">
-      <c r="A481" s="1"/>
-      <c r="B481" s="1"/>
-      <c r="C481" s="1"/>
-      <c r="D481" s="1"/>
-      <c r="E481" s="1"/>
-      <c r="F481" s="1"/>
-      <c r="G481" s="1"/>
-      <c r="H481" s="1"/>
-      <c r="I481" s="1"/>
-      <c r="J481" s="1"/>
-      <c r="K481" s="1"/>
-      <c r="L481" s="1"/>
-      <c r="M481" s="1"/>
-      <c r="N481" s="1"/>
-      <c r="O481" s="1"/>
-      <c r="P481" s="1"/>
-      <c r="Q481" s="1"/>
-    </row>
-    <row r="482" spans="1:17">
-      <c r="A482" s="1"/>
-      <c r="B482" s="1"/>
-      <c r="C482" s="1"/>
-      <c r="D482" s="1"/>
-      <c r="E482" s="1"/>
-      <c r="F482" s="1"/>
-      <c r="G482" s="1"/>
-      <c r="H482" s="1"/>
-      <c r="I482" s="1"/>
-      <c r="J482" s="1"/>
-      <c r="K482" s="1"/>
-      <c r="L482" s="1"/>
-      <c r="M482" s="1"/>
-      <c r="N482" s="1"/>
-      <c r="O482" s="1"/>
-      <c r="P482" s="1"/>
-      <c r="Q482" s="1"/>
-    </row>
-    <row r="483" spans="1:17">
-      <c r="A483" s="1"/>
-      <c r="B483" s="1"/>
-      <c r="C483" s="1"/>
-      <c r="D483" s="1"/>
-      <c r="E483" s="1"/>
-      <c r="F483" s="1"/>
-      <c r="G483" s="1"/>
-      <c r="H483" s="1"/>
-      <c r="I483" s="1"/>
-      <c r="J483" s="1"/>
-      <c r="K483" s="1"/>
-      <c r="L483" s="1"/>
-      <c r="M483" s="1"/>
-      <c r="N483" s="1"/>
-      <c r="O483" s="1"/>
-      <c r="P483" s="1"/>
-      <c r="Q483" s="1"/>
-    </row>
-    <row r="484" spans="1:17">
-      <c r="A484" s="1"/>
-      <c r="B484" s="1"/>
-      <c r="C484" s="1"/>
-      <c r="D484" s="1"/>
-      <c r="E484" s="1"/>
-      <c r="F484" s="1"/>
-      <c r="G484" s="1"/>
-      <c r="H484" s="1"/>
-      <c r="I484" s="1"/>
-      <c r="J484" s="1"/>
-      <c r="K484" s="1"/>
-      <c r="L484" s="1"/>
-      <c r="M484" s="1"/>
-      <c r="N484" s="1"/>
-      <c r="O484" s="1"/>
-      <c r="P484" s="1"/>
-      <c r="Q484" s="1"/>
-    </row>
-    <row r="485" spans="1:17">
-      <c r="A485" s="1"/>
-      <c r="B485" s="1"/>
-      <c r="C485" s="1"/>
-      <c r="D485" s="1"/>
-      <c r="E485" s="1"/>
-      <c r="F485" s="1"/>
-      <c r="G485" s="1"/>
-      <c r="H485" s="1"/>
-      <c r="I485" s="1"/>
-      <c r="J485" s="1"/>
-      <c r="K485" s="1"/>
-      <c r="L485" s="1"/>
-      <c r="M485" s="1"/>
-      <c r="N485" s="1"/>
-      <c r="O485" s="1"/>
-      <c r="P485" s="1"/>
-      <c r="Q485" s="1"/>
-    </row>
-    <row r="486" spans="1:17">
-      <c r="A486" s="1"/>
-      <c r="B486" s="1"/>
-      <c r="C486" s="1"/>
-      <c r="D486" s="1"/>
-      <c r="E486" s="1"/>
-      <c r="F486" s="1"/>
-      <c r="G486" s="1"/>
-      <c r="H486" s="1"/>
-      <c r="I486" s="1"/>
-      <c r="J486" s="1"/>
-      <c r="K486" s="1"/>
-      <c r="L486" s="1"/>
-      <c r="M486" s="1"/>
-      <c r="N486" s="1"/>
-      <c r="O486" s="1"/>
-      <c r="P486" s="1"/>
-      <c r="Q486" s="1"/>
-    </row>
-    <row r="487" spans="1:17">
-      <c r="A487" s="1"/>
-      <c r="B487" s="1"/>
-      <c r="C487" s="1"/>
-      <c r="D487" s="1"/>
-      <c r="E487" s="1"/>
-      <c r="F487" s="1"/>
-      <c r="G487" s="1"/>
-      <c r="H487" s="1"/>
-      <c r="I487" s="1"/>
-      <c r="J487" s="1"/>
-      <c r="K487" s="1"/>
-      <c r="L487" s="1"/>
-      <c r="M487" s="1"/>
-      <c r="N487" s="1"/>
-      <c r="O487" s="1"/>
-      <c r="P487" s="1"/>
-      <c r="Q487" s="1"/>
-    </row>
-    <row r="488" spans="1:17">
-      <c r="A488" s="1"/>
-      <c r="B488" s="1"/>
-      <c r="C488" s="1"/>
-      <c r="D488" s="1"/>
-      <c r="E488" s="1"/>
-      <c r="F488" s="1"/>
-      <c r="G488" s="1"/>
-      <c r="H488" s="1"/>
-      <c r="I488" s="1"/>
-      <c r="J488" s="1"/>
-      <c r="K488" s="1"/>
-      <c r="L488" s="1"/>
-      <c r="M488" s="1"/>
-      <c r="N488" s="1"/>
-      <c r="O488" s="1"/>
-      <c r="P488" s="1"/>
-      <c r="Q488" s="1"/>
-    </row>
-    <row r="489" spans="1:17">
-      <c r="A489" s="1"/>
-      <c r="B489" s="1"/>
-      <c r="C489" s="1"/>
-      <c r="D489" s="1"/>
-      <c r="E489" s="1"/>
-      <c r="F489" s="1"/>
-      <c r="G489" s="1"/>
-      <c r="H489" s="1"/>
-      <c r="I489" s="1"/>
-      <c r="J489" s="1"/>
-      <c r="K489" s="1"/>
-      <c r="L489" s="1"/>
-      <c r="M489" s="1"/>
-      <c r="N489" s="1"/>
-      <c r="O489" s="1"/>
-      <c r="P489" s="1"/>
-      <c r="Q489" s="1"/>
-    </row>
-    <row r="490" spans="1:17">
-      <c r="A490" s="1"/>
-      <c r="B490" s="1"/>
-      <c r="C490" s="1"/>
-      <c r="D490" s="1"/>
-      <c r="E490" s="1"/>
-      <c r="F490" s="1"/>
-      <c r="G490" s="1"/>
-      <c r="H490" s="1"/>
-      <c r="I490" s="1"/>
-      <c r="J490" s="1"/>
-      <c r="K490" s="1"/>
-      <c r="L490" s="1"/>
-      <c r="M490" s="1"/>
-      <c r="N490" s="1"/>
-      <c r="O490" s="1"/>
-      <c r="P490" s="1"/>
-      <c r="Q490" s="1"/>
-    </row>
-    <row r="491" spans="1:17">
-      <c r="A491" s="1"/>
-      <c r="B491" s="1"/>
-      <c r="C491" s="1"/>
-      <c r="D491" s="1"/>
-      <c r="E491" s="1"/>
-      <c r="F491" s="1"/>
-      <c r="G491" s="1"/>
-      <c r="H491" s="1"/>
-      <c r="I491" s="1"/>
-      <c r="J491" s="1"/>
-      <c r="K491" s="1"/>
-      <c r="L491" s="1"/>
-      <c r="M491" s="1"/>
-      <c r="N491" s="1"/>
-      <c r="O491" s="1"/>
-      <c r="P491" s="1"/>
-      <c r="Q491" s="1"/>
-    </row>
-    <row r="492" spans="1:17">
-      <c r="A492" s="1"/>
-      <c r="B492" s="1"/>
-      <c r="C492" s="1"/>
-      <c r="D492" s="1"/>
-      <c r="E492" s="1"/>
-      <c r="F492" s="1"/>
-      <c r="G492" s="1"/>
-      <c r="H492" s="1"/>
-      <c r="I492" s="1"/>
-      <c r="J492" s="1"/>
-      <c r="K492" s="1"/>
-      <c r="L492" s="1"/>
-      <c r="M492" s="1"/>
-      <c r="N492" s="1"/>
-      <c r="O492" s="1"/>
-      <c r="P492" s="1"/>
-      <c r="Q492" s="1"/>
-    </row>
-    <row r="493" spans="1:17">
-      <c r="A493" s="1"/>
-      <c r="B493" s="1"/>
-      <c r="C493" s="1"/>
-      <c r="D493" s="1"/>
-      <c r="E493" s="1"/>
-      <c r="F493" s="1"/>
-      <c r="G493" s="1"/>
-      <c r="H493" s="1"/>
-      <c r="I493" s="1"/>
-      <c r="J493" s="1"/>
-      <c r="K493" s="1"/>
-      <c r="L493" s="1"/>
-      <c r="M493" s="1"/>
-      <c r="N493" s="1"/>
-      <c r="O493" s="1"/>
-      <c r="P493" s="1"/>
-      <c r="Q493" s="1"/>
-    </row>
-    <row r="494" spans="1:17">
-      <c r="A494" s="1"/>
-      <c r="B494" s="1"/>
-      <c r="C494" s="1"/>
-      <c r="D494" s="1"/>
-      <c r="E494" s="1"/>
-      <c r="F494" s="1"/>
-      <c r="G494" s="1"/>
-      <c r="H494" s="1"/>
-      <c r="I494" s="1"/>
-      <c r="J494" s="1"/>
-      <c r="K494" s="1"/>
-      <c r="L494" s="1"/>
-      <c r="M494" s="1"/>
-      <c r="N494" s="1"/>
-      <c r="O494" s="1"/>
-      <c r="P494" s="1"/>
-      <c r="Q494" s="1"/>
-    </row>
-    <row r="495" spans="1:17">
-      <c r="A495" s="1"/>
-      <c r="B495" s="1"/>
-      <c r="C495" s="1"/>
-      <c r="D495" s="1"/>
-      <c r="E495" s="1"/>
-      <c r="F495" s="1"/>
-      <c r="G495" s="1"/>
-      <c r="H495" s="1"/>
-      <c r="I495" s="1"/>
-      <c r="J495" s="1"/>
-      <c r="K495" s="1"/>
-      <c r="L495" s="1"/>
-      <c r="M495" s="1"/>
-      <c r="N495" s="1"/>
-      <c r="O495" s="1"/>
-      <c r="P495" s="1"/>
-      <c r="Q495" s="1"/>
-    </row>
-    <row r="496" spans="1:17">
-      <c r="A496" s="1"/>
-      <c r="B496" s="1"/>
-      <c r="C496" s="1"/>
-      <c r="D496" s="1"/>
-      <c r="E496" s="1"/>
-      <c r="F496" s="1"/>
-      <c r="G496" s="1"/>
-      <c r="H496" s="1"/>
-      <c r="I496" s="1"/>
-      <c r="J496" s="1"/>
-      <c r="K496" s="1"/>
-      <c r="L496" s="1"/>
-      <c r="M496" s="1"/>
-      <c r="N496" s="1"/>
-      <c r="O496" s="1"/>
-      <c r="P496" s="1"/>
-      <c r="Q496" s="1"/>
-    </row>
-    <row r="497" spans="1:17">
-      <c r="A497" s="1"/>
-      <c r="B497" s="1"/>
-      <c r="C497" s="1"/>
-      <c r="D497" s="1"/>
-      <c r="E497" s="1"/>
-      <c r="F497" s="1"/>
-      <c r="G497" s="1"/>
-      <c r="H497" s="1"/>
-      <c r="I497" s="1"/>
-      <c r="J497" s="1"/>
-      <c r="K497" s="1"/>
-      <c r="L497" s="1"/>
-      <c r="M497" s="1"/>
-      <c r="N497" s="1"/>
-      <c r="O497" s="1"/>
-      <c r="P497" s="1"/>
-      <c r="Q497" s="1"/>
-    </row>
-    <row r="498" spans="1:17">
-      <c r="A498" s="1"/>
-      <c r="B498" s="1"/>
-      <c r="C498" s="1"/>
-      <c r="D498" s="1"/>
-      <c r="E498" s="1"/>
-      <c r="F498" s="1"/>
-      <c r="G498" s="1"/>
-      <c r="H498" s="1"/>
-      <c r="I498" s="1"/>
-      <c r="J498" s="1"/>
-      <c r="K498" s="1"/>
-      <c r="L498" s="1"/>
-      <c r="M498" s="1"/>
-      <c r="N498" s="1"/>
-      <c r="O498" s="1"/>
-      <c r="P498" s="1"/>
-      <c r="Q498" s="1"/>
-    </row>
-    <row r="499" spans="1:17">
-      <c r="A499" s="1"/>
-      <c r="B499" s="1"/>
-      <c r="C499" s="1"/>
-      <c r="D499" s="1"/>
-      <c r="E499" s="1"/>
-      <c r="F499" s="1"/>
-      <c r="G499" s="1"/>
-      <c r="H499" s="1"/>
-      <c r="I499" s="1"/>
-      <c r="J499" s="1"/>
-      <c r="K499" s="1"/>
-      <c r="L499" s="1"/>
-      <c r="M499" s="1"/>
-      <c r="N499" s="1"/>
-      <c r="O499" s="1"/>
-      <c r="P499" s="1"/>
-      <c r="Q499" s="1"/>
-    </row>
-    <row r="500" spans="1:17">
-      <c r="A500" s="1"/>
-      <c r="B500" s="1"/>
-      <c r="C500" s="1"/>
-      <c r="D500" s="1"/>
-      <c r="E500" s="1"/>
-      <c r="F500" s="1"/>
-      <c r="G500" s="1"/>
-      <c r="H500" s="1"/>
-      <c r="I500" s="1"/>
-      <c r="J500" s="1"/>
-      <c r="K500" s="1"/>
-      <c r="L500" s="1"/>
-      <c r="M500" s="1"/>
-      <c r="N500" s="1"/>
-      <c r="O500" s="1"/>
-      <c r="P500" s="1"/>
-      <c r="Q500" s="1"/>
-    </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Replace installed company documents with the current ICCT memos and letters.
Campuses that already have templates get those rows removed on update and replaced with the nine seeded documents, including offense-table merge tags and payslip year-to-date.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/resources/templates/employee_salary_upload_template.xlsx
+++ b/resources/templates/employee_salary_upload_template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1385">
   <si>
     <t>employee_name</t>
   </si>
@@ -4125,9 +4125,6 @@
   </si>
   <si>
     <t>CA202505177</t>
-  </si>
-  <si>
-    <t>2026-10-30</t>
   </si>
   <si>
     <t>Villarito, Aprilyn Batosalem</t>
@@ -27816,52 +27813,28 @@
       <c r="C486" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D486" s="1" t="s">
-        <v>1370</v>
-      </c>
+      <c r="D486" s="1"/>
       <c r="E486" s="1"/>
-      <c r="F486" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="G486" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="H486" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="I486" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="J486" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="K486" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="L486" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="M486" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="N486" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="O486" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="P486" s="1" t="s">
-        <v>48</v>
-      </c>
+      <c r="F486" s="1"/>
+      <c r="G486" s="1"/>
+      <c r="H486" s="1"/>
+      <c r="I486" s="1"/>
+      <c r="J486" s="1"/>
+      <c r="K486" s="1"/>
+      <c r="L486" s="1"/>
+      <c r="M486" s="1"/>
+      <c r="N486" s="1"/>
+      <c r="O486" s="1"/>
+      <c r="P486" s="1"/>
       <c r="Q486" s="1"/>
       <c r="R486" s="1"/>
     </row>
     <row r="487" spans="1:18">
       <c r="A487" s="1" t="s">
+        <v>1370</v>
+      </c>
+      <c r="B487" s="1" t="s">
         <v>1371</v>
-      </c>
-      <c r="B487" s="1" t="s">
-        <v>1372</v>
       </c>
       <c r="C487" s="1" t="s">
         <v>38</v>
@@ -27906,10 +27879,10 @@
     </row>
     <row r="488" spans="1:18">
       <c r="A488" s="1" t="s">
+        <v>1372</v>
+      </c>
+      <c r="B488" s="1" t="s">
         <v>1373</v>
-      </c>
-      <c r="B488" s="1" t="s">
-        <v>1374</v>
       </c>
       <c r="C488" s="1" t="s">
         <v>38</v>
@@ -27954,16 +27927,16 @@
     </row>
     <row r="489" spans="1:18">
       <c r="A489" s="1" t="s">
+        <v>1374</v>
+      </c>
+      <c r="B489" s="1" t="s">
         <v>1375</v>
       </c>
-      <c r="B489" s="1" t="s">
+      <c r="C489" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D489" s="1" t="s">
         <v>1376</v>
-      </c>
-      <c r="C489" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D489" s="1" t="s">
-        <v>1377</v>
       </c>
       <c r="E489" s="1"/>
       <c r="F489" s="1" t="s">
@@ -28002,10 +27975,10 @@
     </row>
     <row r="490" spans="1:18">
       <c r="A490" s="1" t="s">
+        <v>1377</v>
+      </c>
+      <c r="B490" s="1" t="s">
         <v>1378</v>
-      </c>
-      <c r="B490" s="1" t="s">
-        <v>1379</v>
       </c>
       <c r="C490" s="1" t="s">
         <v>38</v>
@@ -28028,16 +28001,16 @@
     </row>
     <row r="491" spans="1:18">
       <c r="A491" s="1" t="s">
+        <v>1379</v>
+      </c>
+      <c r="B491" s="1" t="s">
         <v>1380</v>
       </c>
-      <c r="B491" s="1" t="s">
+      <c r="C491" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D491" s="1" t="s">
         <v>1381</v>
-      </c>
-      <c r="C491" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D491" s="1" t="s">
-        <v>1382</v>
       </c>
       <c r="E491" s="1"/>
       <c r="F491" s="1" t="s">
@@ -28076,16 +28049,16 @@
     </row>
     <row r="492" spans="1:18">
       <c r="A492" s="1" t="s">
+        <v>1382</v>
+      </c>
+      <c r="B492" s="1" t="s">
         <v>1383</v>
       </c>
-      <c r="B492" s="1" t="s">
+      <c r="C492" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D492" s="1" t="s">
         <v>1384</v>
-      </c>
-      <c r="C492" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D492" s="1" t="s">
-        <v>1385</v>
       </c>
       <c r="E492" s="1"/>
       <c r="F492" s="1" t="s">

</xml_diff>